<commit_message>
Fixed issue with parsing 4-digit dates as if they were 2-digit powerof10 dates, though powerof10 changed now anyway.
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4CF9A8-7B86-41A5-896F-0FD3BFAF7B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D6EBD6-30F9-4D15-826A-CA386512E9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="92">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -107,9 +107,6 @@
     <t>Add known performances here (e.g. for road events) that predate powerof10 and are missing from the official C&amp;C T&amp;F records</t>
   </si>
   <si>
-    <t>14 Oct ????</t>
-  </si>
-  <si>
     <t>Mark Vile clipping ---&gt;</t>
   </si>
   <si>
@@ -312,6 +309,12 @@
   </si>
   <si>
     <t>https://www.valenciaciudaddelrunning.com/en/marathon/2025-marathon-ranking/</t>
+  </si>
+  <si>
+    <t>14 Oct 1979</t>
+  </si>
+  <si>
+    <t>also listed here with year</t>
   </si>
 </sst>
 </file>
@@ -945,7 +948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6262A1C6-2E08-4627-9589-5880845FD58A}">
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49" style="1" bestFit="1" customWidth="1"/>
@@ -954,12 +957,12 @@
     <col min="12" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="6" t="s">
         <v>14</v>
@@ -992,7 +995,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>8</v>
@@ -1022,24 +1025,24 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>4</v>
@@ -1048,24 +1051,27 @@
         <v>3</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="G6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>4</v>
@@ -1074,102 +1080,102 @@
         <v>3</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="I9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G9" s="1" t="s">
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>4</v>
@@ -1178,24 +1184,24 @@
         <v>3</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="D11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>4</v>
@@ -1204,24 +1210,24 @@
         <v>3</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>4</v>
@@ -1230,143 +1236,143 @@
         <v>3</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="K13" s="1" t="s">
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
+      <c r="D14" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K14" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K15" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
+      <c r="F16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="H16" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
@@ -1382,8 +1388,9 @@
     <hyperlink ref="E4" r:id="rId1" xr:uid="{DA518F53-48F6-4384-B523-77D886998775}"/>
     <hyperlink ref="H16" r:id="rId2" xr:uid="{5AFD5061-E0E2-4CD1-893D-97AB7D024121}"/>
     <hyperlink ref="H17" r:id="rId3" xr:uid="{8DC9337C-503C-44C4-BA48-F245BD1982AF}"/>
+    <hyperlink ref="L5" r:id="rId4" xr:uid="{F09E7A36-9A19-457D-8AA2-2555BD6668C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding recent performances by GC which should be MV65 records
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D6EBD6-30F9-4D15-826A-CA386512E9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8074ABB1-5BF9-4FE8-997A-07654D9D1306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="1700" yWindow="1050" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="107">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -315,6 +315,51 @@
   </si>
   <si>
     <t>also listed here with year</t>
+  </si>
+  <si>
+    <t>Giulio Cinque</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>15.2</t>
+  </si>
+  <si>
+    <t>31.5</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>EMAC league</t>
+  </si>
+  <si>
+    <t>3 Jun 2026</t>
+  </si>
+  <si>
+    <t>1 Jul 2026</t>
+  </si>
+  <si>
+    <t>HM</t>
+  </si>
+  <si>
+    <t>Cambridge Half Marathon</t>
+  </si>
+  <si>
+    <t>Cambridge EMAC league</t>
+  </si>
+  <si>
+    <t>Kings Lynn EMAC league</t>
+  </si>
+  <si>
+    <t>1:38:07</t>
+  </si>
+  <si>
+    <t>8 Mar 2026</t>
+  </si>
+  <si>
+    <t>https://emac.org.uk/track-field-league/2026-track-field-league/</t>
   </si>
 </sst>
 </file>
@@ -648,6 +693,138 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>527208</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>133365</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7172F209-D47E-6561-4375-AFC0BC95AECE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18370550" y="3168650"/>
+          <a:ext cx="3067208" cy="285765"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>488950</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>28534</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>45084</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>88949</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE072655-4411-2E22-2E37-16CD7776BF61}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18859500" y="3032084"/>
+          <a:ext cx="2731134" cy="219165"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>457578</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>362529</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>79383</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20E00FDA-2D95-9264-BA01-8F52957A8A95}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17558128" y="2876550"/>
+          <a:ext cx="2444951" cy="206383"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1375,6 +1552,90 @@
         <v>84</v>
       </c>
     </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
     <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
     </row>
@@ -1389,8 +1650,10 @@
     <hyperlink ref="H16" r:id="rId2" xr:uid="{5AFD5061-E0E2-4CD1-893D-97AB7D024121}"/>
     <hyperlink ref="H17" r:id="rId3" xr:uid="{8DC9337C-503C-44C4-BA48-F245BD1982AF}"/>
     <hyperlink ref="L5" r:id="rId4" xr:uid="{F09E7A36-9A19-457D-8AA2-2555BD6668C1}"/>
+    <hyperlink ref="H18" r:id="rId5" xr:uid="{D5CD19BD-71B8-4DEE-8EBC-E2E69408E82A}"/>
+    <hyperlink ref="H19" r:id="rId6" xr:uid="{928A744B-E999-4747-93B8-666BBDBF86D5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Inserting GC's middle initial to match po10 name, to avoid duplication in record table
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8074ABB1-5BF9-4FE8-997A-07654D9D1306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5934BED4-33E3-440B-ACE9-0139A6EE620B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1700" yWindow="1050" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="108">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -317,9 +317,6 @@
     <t>also listed here with year</t>
   </si>
   <si>
-    <t>Giulio Cinque</t>
-  </si>
-  <si>
     <t>100</t>
   </si>
   <si>
@@ -360,6 +357,12 @@
   </si>
   <si>
     <t>https://emac.org.uk/track-field-league/2026-track-field-league/</t>
+  </si>
+  <si>
+    <t>Giulio A Cinque</t>
+  </si>
+  <si>
+    <t>EMAC league; using po10 name with initial to avoid duplication</t>
   </si>
 </sst>
 </file>
@@ -1554,22 +1557,22 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="G18" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>4</v>
@@ -1578,27 +1581,27 @@
         <v>77</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>96</v>
-      </c>
       <c r="G19" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>4</v>
@@ -1607,24 +1610,24 @@
         <v>77</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="D20" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="F20" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>4</v>
@@ -1633,7 +1636,7 @@
         <v>77</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added some records for E S-W as advised by email
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5934BED4-33E3-440B-ACE9-0139A6EE620B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7660B31-B80C-4F9F-9E68-A531DBB114E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="1130" yWindow="300" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="122">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -363,6 +363,48 @@
   </si>
   <si>
     <t>EMAC league; using po10 name with initial to avoid duplication</t>
+  </si>
+  <si>
+    <t>Eunice Stewart-Wallace</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/c80cac89-1b45-49ee-bf95-ebfe940ba266</t>
+  </si>
+  <si>
+    <t>HJ</t>
+  </si>
+  <si>
+    <t>1.58</t>
+  </si>
+  <si>
+    <t>26 Apr 2026</t>
+  </si>
+  <si>
+    <t>Cambridge EYAL</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/a43a7a1b-ff84-4da9-89e1-0bf5d103a29f</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>42.1</t>
+  </si>
+  <si>
+    <t>31 May 2026</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/1cad6874-57f2-44fa-b6e4-29f66223d6b5</t>
+  </si>
+  <si>
+    <t>Bury St Edmunds EAT&amp;FL</t>
+  </si>
+  <si>
+    <t>U16</t>
+  </si>
+  <si>
+    <t>From email</t>
   </si>
 </sst>
 </file>
@@ -1132,7 +1174,9 @@
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="10" width="17.36328125" style="1" customWidth="1"/>
+    <col min="2" max="3" width="17.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7265625" style="1" customWidth="1"/>
+    <col min="5" max="10" width="17.36328125" style="1" customWidth="1"/>
     <col min="11" max="11" width="30.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="9.08984375" style="1"/>
   </cols>
@@ -1637,6 +1681,70 @@
       </c>
       <c r="K20" s="1" t="s">
         <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
@@ -1655,8 +1763,12 @@
     <hyperlink ref="L5" r:id="rId4" xr:uid="{F09E7A36-9A19-457D-8AA2-2555BD6668C1}"/>
     <hyperlink ref="H18" r:id="rId5" xr:uid="{D5CD19BD-71B8-4DEE-8EBC-E2E69408E82A}"/>
     <hyperlink ref="H19" r:id="rId6" xr:uid="{928A744B-E999-4747-93B8-666BBDBF86D5}"/>
+    <hyperlink ref="E21" r:id="rId7" xr:uid="{87A66CE3-B38D-4C01-9FC8-9B5FBCD21198}"/>
+    <hyperlink ref="H21" r:id="rId8" xr:uid="{E98CC6FD-6BDC-42E6-AB65-1946CD28BF45}"/>
+    <hyperlink ref="E22" r:id="rId9" xr:uid="{D207200A-9073-4A0B-8AF3-2A6DB1D2B1CD}"/>
+    <hyperlink ref="H22" r:id="rId10" xr:uid="{3A25B3C5-0B4B-499C-907C-6232CB2EC938}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added all recent records from Google Drive sheet validated by Stu Dunlop
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7660B31-B80C-4F9F-9E68-A531DBB114E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF3B0F8-3537-46EB-BEDC-D999B61CDA78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1130" yWindow="300" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="204">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -405,6 +405,252 @@
   </si>
   <si>
     <t>From email</t>
+  </si>
+  <si>
+    <t>Stefanie Godfrey</t>
+  </si>
+  <si>
+    <t>1:32:01</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/d290b5e6-c2da-4d2a-b095-d00ae8b78f4e</t>
+  </si>
+  <si>
+    <t>From self-report form validated by Stu Dunlop</t>
+  </si>
+  <si>
+    <t>Miguel Branco</t>
+  </si>
+  <si>
+    <t>V45</t>
+  </si>
+  <si>
+    <t>33:53</t>
+  </si>
+  <si>
+    <t>73:10</t>
+  </si>
+  <si>
+    <t>16:13</t>
+  </si>
+  <si>
+    <t>Battersea Park, London</t>
+  </si>
+  <si>
+    <t>Cambridge</t>
+  </si>
+  <si>
+    <t>14 Feb 2026</t>
+  </si>
+  <si>
+    <t>25 Apr 2026</t>
+  </si>
+  <si>
+    <t>Darren Preston</t>
+  </si>
+  <si>
+    <t>V50</t>
+  </si>
+  <si>
+    <t>16:25</t>
+  </si>
+  <si>
+    <t>Kingsley Mid Cheshire 5K</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/56c16c5b-7247-4b39-b572-b60ca2c431de</t>
+  </si>
+  <si>
+    <t>22 May 2026</t>
+  </si>
+  <si>
+    <t>Martin Kilduff</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/a35bbe63-635c-4ac8-b40d-035383ffc815</t>
+  </si>
+  <si>
+    <t>Mile</t>
+  </si>
+  <si>
+    <t>V75</t>
+  </si>
+  <si>
+    <t>6:53.5</t>
+  </si>
+  <si>
+    <t>London</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/5f4c9b08-24d2-41e8-ada4-f43bb0276356</t>
+  </si>
+  <si>
+    <t>4:11:01</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/4c6db59a-49fa-40e0-83b3-0b09a70d34e3</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/0eabae36-e4f0-40a7-9b85-3b2e924e5468</t>
+  </si>
+  <si>
+    <t>David Van Den Bergh</t>
+  </si>
+  <si>
+    <t>1.5</t>
+  </si>
+  <si>
+    <t>27 Mar 2026</t>
+  </si>
+  <si>
+    <t>14.7</t>
+  </si>
+  <si>
+    <t>9.08</t>
+  </si>
+  <si>
+    <t>TJ</t>
+  </si>
+  <si>
+    <t>4.22</t>
+  </si>
+  <si>
+    <t>LJ</t>
+  </si>
+  <si>
+    <t>70.9</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>55.18</t>
+  </si>
+  <si>
+    <t>300HM60</t>
+  </si>
+  <si>
+    <t>21 Feb 2026</t>
+  </si>
+  <si>
+    <t>14 Jun 2026</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/eb2423c7-48c8-48b1-ab5e-ccb11ce8b4f1</t>
+  </si>
+  <si>
+    <t>European Masters, Torun, Poland</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/3bbabf78-c0f4-440e-90ff-6d08113f7cf7</t>
+  </si>
+  <si>
+    <t>BMAF Champs, Lee Valley</t>
+  </si>
+  <si>
+    <t>EMAC Champs, Sandy</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/5d090524-eb52-474f-87c0-571e8190efbb</t>
+  </si>
+  <si>
+    <t>Brielle Chiy</t>
+  </si>
+  <si>
+    <t>Sarah Abramson</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/ce35a2a0-1863-4e95-b010-c75b1ce70fde</t>
+  </si>
+  <si>
+    <t>Ware</t>
+  </si>
+  <si>
+    <t>U18</t>
+  </si>
+  <si>
+    <t>HT3K</t>
+  </si>
+  <si>
+    <t>49.76</t>
+  </si>
+  <si>
+    <t>49.83</t>
+  </si>
+  <si>
+    <t>41.4</t>
+  </si>
+  <si>
+    <t>20 May 2026</t>
+  </si>
+  <si>
+    <t>19 Apr 2026</t>
+  </si>
+  <si>
+    <t>21 Jun 2026</t>
+  </si>
+  <si>
+    <t>St Ives</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/bca25c88-6862-4617-b068-213f15703fb4</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/09550bca-d312-445f-8a91-e7e3387958b0</t>
+  </si>
+  <si>
+    <t>HT4K</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/e370d06f-883c-47af-a97f-1bb59e2cbbb1</t>
+  </si>
+  <si>
+    <t>Stamford</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/48b83e10-7422-4ea8-a37b-8902b032cdc5</t>
+  </si>
+  <si>
+    <t>2:24:29</t>
+  </si>
+  <si>
+    <t>30K</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/720bdca2-0180-40ea-a88a-e2cb939ab971</t>
+  </si>
+  <si>
+    <t>15 Feb 2026</t>
+  </si>
+  <si>
+    <t>PenIM60</t>
+  </si>
+  <si>
+    <t>31 Mar 2026</t>
+  </si>
+  <si>
+    <t>2384</t>
+  </si>
+  <si>
+    <t>30.6</t>
+  </si>
+  <si>
+    <t>28 Jul 2026</t>
+  </si>
+  <si>
+    <t>Peterborough EMAC</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/eb6aec51-c890-40c7-ac3c-b360b203a3a7</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/9233943c-36a5-40b2-9ffd-5baec1e29f33</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/ac121869-898d-4916-8778-bd20a2a3bedb</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/bc3909e2-2a08-4893-b32c-5765e236bb6f</t>
   </si>
 </sst>
 </file>
@@ -1171,22 +1417,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6262A1C6-2E08-4627-9589-5880845FD58A}">
   <dimension ref="A1:L59"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7265625" style="1" customWidth="1"/>
-    <col min="5" max="10" width="17.36328125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="30.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.08984375" style="1"/>
+    <col min="2" max="3" width="17.3828125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.69140625" style="1" customWidth="1"/>
+    <col min="5" max="10" width="17.3828125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="30.4609375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.07421875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="17.600000000000001" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="6" t="s">
         <v>14</v>
@@ -1219,7 +1465,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>8</v>
@@ -1249,7 +1495,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1281,7 +1527,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1307,7 +1553,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
@@ -1333,7 +1579,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1359,7 +1605,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>47</v>
       </c>
@@ -1385,7 +1631,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>53</v>
       </c>
@@ -1411,7 +1657,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>57</v>
       </c>
@@ -1437,7 +1683,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>61</v>
       </c>
@@ -1463,7 +1709,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1489,7 +1735,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>69</v>
       </c>
@@ -1515,7 +1761,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>73</v>
       </c>
@@ -1541,7 +1787,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>80</v>
       </c>
@@ -1570,7 +1816,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>86</v>
       </c>
@@ -1599,7 +1845,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>93</v>
       </c>
@@ -1628,7 +1874,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>94</v>
       </c>
@@ -1657,7 +1903,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>103</v>
       </c>
@@ -1683,7 +1929,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>111</v>
       </c>
@@ -1715,7 +1961,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
         <v>116</v>
       </c>
@@ -1747,10 +1993,601 @@
         <v>121</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B23" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B24" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B25" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B26" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B27" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B28" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B29" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B30" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B31" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
-    </row>
-    <row r="59" spans="1:1" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B33" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B34" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B35" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B36" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B37" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B38" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B39" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B40" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B41" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="14.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>0</v>
       </c>
@@ -1767,8 +2604,16 @@
     <hyperlink ref="H21" r:id="rId8" xr:uid="{E98CC6FD-6BDC-42E6-AB65-1946CD28BF45}"/>
     <hyperlink ref="E22" r:id="rId9" xr:uid="{D207200A-9073-4A0B-8AF3-2A6DB1D2B1CD}"/>
     <hyperlink ref="H22" r:id="rId10" xr:uid="{3A25B3C5-0B4B-499C-907C-6232CB2EC938}"/>
+    <hyperlink ref="H23" r:id="rId11" xr:uid="{C5C3BB8C-3627-4760-8AE8-9DD0B04375EB}"/>
+    <hyperlink ref="E39" r:id="rId12" xr:uid="{C9BF6B4A-A344-424F-A454-3B5E1B7C4882}"/>
+    <hyperlink ref="E40" r:id="rId13" xr:uid="{35A917CB-3C8E-4635-AC78-C7321890E862}"/>
+    <hyperlink ref="H41" r:id="rId14" xr:uid="{B025A92E-5819-4C31-8F20-4DA02D570C34}"/>
+    <hyperlink ref="H40" r:id="rId15" xr:uid="{E79746ED-0ED9-4730-8A4E-CC6D57FF41B9}"/>
+    <hyperlink ref="H26" r:id="rId16" xr:uid="{86A716B5-319A-4988-BBB0-A974619BF2CA}"/>
+    <hyperlink ref="H25" r:id="rId17" xr:uid="{5989654A-8A56-4C21-B7F2-952EC54B8FF7}"/>
+    <hyperlink ref="E27" r:id="rId18" xr:uid="{3394B413-0143-4554-8881-5A939C20DACD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId19"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding LW hurdles results from SD
</commit_message>
<xml_diff>
--- a/CnC_known_historical.xlsx
+++ b/CnC_known_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\powerof10-tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\powerof10-tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF3B0F8-3537-46EB-BEDC-D999B61CDA78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96D7E93-B2F1-40A9-8DD2-4E3BC4F35429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
+    <workbookView xWindow="1130" yWindow="300" windowWidth="23900" windowHeight="13350" xr2:uid="{DE35B28A-4815-4142-AF1E-480F61EDA5DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Other" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="216">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -651,6 +651,42 @@
   </si>
   <si>
     <t>https://www.powerof10.uk/Home/Results/bc3909e2-2a08-4893-b32c-5765e236bb6f</t>
+  </si>
+  <si>
+    <t>Leah Wagstaff</t>
+  </si>
+  <si>
+    <t>U20</t>
+  </si>
+  <si>
+    <t>11 Jul 2026</t>
+  </si>
+  <si>
+    <t>20 Jun 2026</t>
+  </si>
+  <si>
+    <t>Birmingham - English Schools Champs</t>
+  </si>
+  <si>
+    <t>Birmingham - GB Champs</t>
+  </si>
+  <si>
+    <t>13.73</t>
+  </si>
+  <si>
+    <t>13.8</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Athlete/48806685-7c3b-4e29-adaf-e005cb5e6a19</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/082e2d04-58ee-42d7-a485-59a3587ebf55</t>
+  </si>
+  <si>
+    <t>https://www.powerof10.uk/Home/Results/02bc01fd-7392-4b36-a9fe-8c4fbcdbef97</t>
+  </si>
+  <si>
+    <t>100HW</t>
   </si>
 </sst>
 </file>
@@ -1417,22 +1453,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6262A1C6-2E08-4627-9589-5880845FD58A}">
   <dimension ref="A1:L59"/>
-  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.3828125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.69140625" style="1" customWidth="1"/>
-    <col min="5" max="10" width="17.3828125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="30.4609375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.07421875" style="1"/>
+    <col min="2" max="3" width="17.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7265625" style="1" customWidth="1"/>
+    <col min="5" max="10" width="17.36328125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="30.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="6" t="s">
         <v>14</v>
@@ -1465,7 +1501,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>8</v>
@@ -1495,7 +1531,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1527,7 +1563,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1553,7 +1589,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
@@ -1579,7 +1615,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>37</v>
       </c>
@@ -1605,7 +1641,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>47</v>
       </c>
@@ -1631,7 +1667,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>53</v>
       </c>
@@ -1657,7 +1693,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>57</v>
       </c>
@@ -1683,7 +1719,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>61</v>
       </c>
@@ -1709,7 +1745,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1735,7 +1771,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>69</v>
       </c>
@@ -1761,7 +1797,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>73</v>
       </c>
@@ -1787,7 +1823,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>80</v>
       </c>
@@ -1816,7 +1852,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>86</v>
       </c>
@@ -1845,7 +1881,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>93</v>
       </c>
@@ -1874,7 +1910,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>94</v>
       </c>
@@ -1903,7 +1939,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>103</v>
       </c>
@@ -1929,7 +1965,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>111</v>
       </c>
@@ -1961,7 +1997,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>116</v>
       </c>
@@ -1993,7 +2029,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>123</v>
       </c>
@@ -2022,7 +2058,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>128</v>
       </c>
@@ -2051,7 +2087,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
         <v>129</v>
       </c>
@@ -2080,7 +2116,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>130</v>
       </c>
@@ -2109,7 +2145,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>137</v>
       </c>
@@ -2141,7 +2177,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>145</v>
       </c>
@@ -2173,7 +2209,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>148</v>
       </c>
@@ -2205,7 +2241,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
         <v>152</v>
       </c>
@@ -2237,7 +2273,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>154</v>
       </c>
@@ -2269,7 +2305,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="1" t="s">
         <v>155</v>
@@ -2302,7 +2338,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>159</v>
       </c>
@@ -2334,7 +2370,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
         <v>157</v>
       </c>
@@ -2366,7 +2402,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>161</v>
       </c>
@@ -2398,7 +2434,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
         <v>177</v>
       </c>
@@ -2430,7 +2466,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>178</v>
       </c>
@@ -2462,7 +2498,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
         <v>179</v>
       </c>
@@ -2494,7 +2530,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
         <v>190</v>
       </c>
@@ -2522,8 +2558,11 @@
       <c r="J39" s="1" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="K39" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>197</v>
       </c>
@@ -2555,7 +2594,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B41" s="1" t="s">
         <v>196</v>
       </c>
@@ -2587,7 +2626,71 @@
         <v>125</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="14.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>0</v>
       </c>
@@ -2612,8 +2715,10 @@
     <hyperlink ref="H26" r:id="rId16" xr:uid="{86A716B5-319A-4988-BBB0-A974619BF2CA}"/>
     <hyperlink ref="H25" r:id="rId17" xr:uid="{5989654A-8A56-4C21-B7F2-952EC54B8FF7}"/>
     <hyperlink ref="E27" r:id="rId18" xr:uid="{3394B413-0143-4554-8881-5A939C20DACD}"/>
+    <hyperlink ref="H42" r:id="rId19" xr:uid="{0AFBFB3D-A621-49B6-9AED-DFB855EAF16A}"/>
+    <hyperlink ref="H43" r:id="rId20" xr:uid="{1469BDE7-0674-474D-A6CE-8CD56D1EF9BC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId19"/>
+  <drawing r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>